<commit_message>
update excel kb 19Okt2026
</commit_message>
<xml_diff>
--- a/Excels/Knowledge Base.xlsx
+++ b/Excels/Knowledge Base.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://itservicewn.sharepoint.com/sites/VODAFONEVIER/Freigegebene Dokumente/General/FAQ/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Zeyuan.Sun\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EE63BB4F-29FE-4BDB-B71C-0B8AA884EBA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C97794A-0794-40C9-BE7B-FB1CC11B5996}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="81">
   <si>
     <t>Zusätzliche Informationen / Wissensdatenbank für den FAQ-Bot</t>
   </si>
@@ -126,9 +126,6 @@
     <t>Gasversorgung – Bioerdgas</t>
   </si>
   <si>
-    <t>Anfragen zum Bezug von Bioerdgas/Biogas sowie zu einem benötigten Biogas-Nachweis müssen individuell durch den zuständigen Fachbereich geprüft werden. Dies betrifft beispielsweise die Frage, ob Bioerdgas über die Stadtwerke Waiblingen bezogen werden kann, wie ein Bezug möglich ist oder ob ein von einer Stadt bzw. Behörde geforderter Nachweis für Biogas ausgestellt werden kann. Schreiben Sie hierzu gerne eine E-Mail an vertrieb@stadtwerke-waiblingen.de oder bleiben sie in der Leitung, um mit einem Mitarbeiter verbunden zu werden.</t>
-  </si>
-  <si>
     <t>Lieferantenwechsel – Widerruf Fremdvertrag</t>
   </si>
   <si>
@@ -141,10 +138,45 @@
     <t>Ein bereits angestoßener Tarifwechsel kann widerrufen werden. Der Widerruf muss schriftlich erfolgen. Hierfür können Sie eine E-Mail an vertrieb@stadtwerke-waiblingen.de senden oder den Widerrufs-Button auf der Website nutzen. Nach Eingang des Widerrufs wird das Anliegen geprüft und bearbeitet.</t>
   </si>
   <si>
-    <t>Elektromobilität – Autostromvertrag und Ladekarte</t>
-  </si>
-  <si>
-    <t>Bei Abschluss eines Autostrom-Vertrags bei den Stadtwerken Waiblingen kann der Kunde auf Wunsch eine Ladekarte erhalten. Informationen zum Autostrom-Vertrag und zur Ladekarte sind auf der Website der Stadtwerke Waiblingen verfügbar.</t>
+    <t>Elektromobilität – Autostromvertrag</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(Information wie der Kunde vorgehen muss, wird noch definiert - Pembe)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: Ja, einen Autostromvertrag können Sie bei uns abschließen. Den Antrag finden Sie auf unserer Homepage im Bereich E-Mobilität. Bitte füllen Sie das Formular aus und senden Sie es anschließend unterschrieben per E-Mail an vertrieb@stadtwerke-waiblingen.de. Bei Fragen helfen wir Ihnen gerne weiter.</t>
+    </r>
+  </si>
+  <si>
+    <t>Elektromobilität - Ladekarte</t>
+  </si>
+  <si>
+    <t>Bei Abschluss eines Autostrom-Vertrags bei den Stadtwerken Waiblingen kann der Kunde auf Wunsch eine Ladekarte erhalten.</t>
   </si>
   <si>
     <t>Stammdaten – Namensänderung nach Heirat</t>
@@ -165,6 +197,12 @@
     <t>Ist aufgrund des Todesfalls eines Ehe- oder Lebenspartners eine Namensänderung erforderlich, muss die Änderung den Stadtwerken Waiblingen schriftlich mitgeteilt werden. Die Mitteilung kann per E-Mail oder Post erfolgen.</t>
   </si>
   <si>
+    <t xml:space="preserve">Stammdaten - Kontaktdaten ändern </t>
+  </si>
+  <si>
+    <t>Eine Änderung der Kontaktdaten wie Telefonnummer oder E-Mailadresse muss den Stadtwerken Waiblingen schriftlich mitgeteilt werden.</t>
+  </si>
+  <si>
     <t>SEPA – Änderung der Bankverbindung</t>
   </si>
   <si>
@@ -247,13 +285,64 @@
   </si>
   <si>
     <t>Können Sie eine offene Jahresverbrauchsabrechnung nicht auf einmal bezahlen, kann eine Ratenzahlungsvereinbarung mit einer Laufzeit von maximal sechs Monaten beantragt werden. Der Ratenvertrag kann jeweils zum 1. oder zum 15. eines Monats beginnen. Möchten Sie eine Ratenzahlung vereinbaren, senden Sie uns bitte eine E-Mail an info@stadtwerke-waiblingen.de und teilen Sie uns die gewünschten Angaben zur Ratenzahlung mit. Ihr Antrag wird anschließend geprüft. Bei Bewilligung erhalten Sie den Ratenzahlungsvertrag in den nächsten Tagen in Papierform.</t>
+  </si>
+  <si>
+    <t>Umzug - bereits eingezogen</t>
+  </si>
+  <si>
+    <t>Wenn der Kunde bereits in die neue Wohnung eingezogen ist und seinen Einzug noch nicht gemeldet hat, soll er seinen Einzug über das Umzugsformular auf der Homepage melden.</t>
+  </si>
+  <si>
+    <t>Umzug - Zukünftiger Umzug</t>
+  </si>
+  <si>
+    <t>Wenn der Kunde erst zukünftig einzieht, soll der geplante Einzug ebenfalls über das Umzugsformular auf der Homepage gemeldet werden. Hier benötigen wir dann die Zählerstände zum Tag der Schlüsselübergabe.</t>
+  </si>
+  <si>
+    <t>Rechnung - fehlt</t>
+  </si>
+  <si>
+    <t>Wenn wir Ihren Zählerstand vorliegen haben, wird  die Rechnung zeitnah von uns erstellt. Falls uns ihr Zählerstand noch nicht vorliegt, teilen Sie uns diesen bitte unter zaehlerstand@stadtwerke-waiblingen.de mit</t>
+  </si>
+  <si>
+    <t>Notfallnummern - Strom, Gas, Wasser, Fernwärme</t>
+  </si>
+  <si>
+    <t>Wenn Sie eine Störung im Versorgungsnetz feststellen, können Sie sich rund um die Uhr an unseren Entstörungsdienst wenden. Der Entstörungsdienst ist 24 Stunden am Tag und an 365 Tagen im Jahr erreichbar.
+Wenn Sie einen Stromausfall oder eine andere Störung der Stromversorgung haben, melden Sie sich bitte unter 07151 131-301.
+Wenn Sie Gasgeruch wahrnehmen, einen Gasaustritt vermuten oder eine andere Störung der Gasversorgung feststellen, melden Sie sich bitte unter 07151 131-601.
+Wenn Sie kein Wasser haben, einen Rohrbruch oder eine andere Störung der Wasserversorgung feststellen, melden Sie sich bitte unter 07151 131-401.
+Wenn Ihre Fernwärmeversorgung ausgefallen ist oder Sie eine andere Störung im Fernwärmenetz feststellen, melden Sie sich bitte unter 07151 131-501.
+Die Notfallnummern sind ausschließlich für Störungen im jeweiligen Versorgungsnetz vorgesehen.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Anfragen zum Bezug von Bioerdgas/Biogas sowie zu einem benötigten Biogas-Nachweis müssen individuell durch den zuständigen Fachbereich geprüft werden. Dies betrifft beispielsweise die Frage, ob Bioerdgas über die Stadtwerke Waiblingen bezogen werden kann, wie ein Bezug möglich ist oder ob ein von einer Stadt bzw. Behörde geforderter Nachweis für Biogas ausgestellt werden kann. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(Kein Hinweis auf die E-Mailadresse geben).</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -287,7 +376,33 @@
       <sz val="11"/>
       <color rgb="FF242424"/>
       <name val="Aptos Narrow"/>
-      <charset val="1"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="5">
@@ -316,7 +431,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -363,11 +478,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -394,7 +524,22 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -413,9 +558,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 – 2022-Design">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 – 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -453,7 +598,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 – 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -559,7 +704,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 – 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -701,7 +846,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -709,22 +854,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:D40"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <dimension ref="B2:D43"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="4.42578125" customWidth="1"/>
-    <col min="2" max="2" width="43.28515625" customWidth="1"/>
-    <col min="3" max="3" width="170.140625" customWidth="1"/>
+    <col min="1" max="1" width="4.453125" customWidth="1"/>
+    <col min="2" max="2" width="43.26953125" customWidth="1"/>
+    <col min="3" max="3" width="170.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:4" ht="23.25" customHeight="1">
+    <row r="2" spans="2:4" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B2" s="6" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="5"/>
       <c r="D2" s="7"/>
     </row>
-    <row r="4" spans="2:4" ht="26.25" customHeight="1">
+    <row r="4" spans="2:4" ht="26.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B4" s="2" t="s">
         <v>1</v>
       </c>
@@ -732,7 +877,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="2:4" ht="30">
+    <row r="5" spans="2:4" ht="29" x14ac:dyDescent="0.35">
       <c r="B5" s="3" t="s">
         <v>3</v>
       </c>
@@ -740,7 +885,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="2:4" ht="30">
+    <row r="6" spans="2:4" ht="29" x14ac:dyDescent="0.35">
       <c r="B6" s="3" t="s">
         <v>5</v>
       </c>
@@ -748,7 +893,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="2:4" ht="30">
+    <row r="7" spans="2:4" ht="29" x14ac:dyDescent="0.35">
       <c r="B7" s="3" t="s">
         <v>7</v>
       </c>
@@ -756,7 +901,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="2:4" ht="75">
+    <row r="8" spans="2:4" ht="43.5" x14ac:dyDescent="0.35">
       <c r="B8" s="3" t="s">
         <v>9</v>
       </c>
@@ -764,7 +909,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="2:4" ht="30">
+    <row r="9" spans="2:4" ht="29" x14ac:dyDescent="0.35">
       <c r="B9" s="3" t="s">
         <v>11</v>
       </c>
@@ -772,7 +917,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="2:4">
+    <row r="10" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B10" s="3" t="s">
         <v>13</v>
       </c>
@@ -780,7 +925,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="11" spans="2:4" ht="60">
+    <row r="11" spans="2:4" ht="43.5" x14ac:dyDescent="0.35">
       <c r="B11" s="3" t="s">
         <v>15</v>
       </c>
@@ -788,7 +933,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="2:4" ht="30">
+    <row r="12" spans="2:4" ht="29" x14ac:dyDescent="0.35">
       <c r="B12" s="3" t="s">
         <v>17</v>
       </c>
@@ -796,7 +941,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="13" spans="2:4" ht="30">
+    <row r="13" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B13" s="3" t="s">
         <v>19</v>
       </c>
@@ -804,23 +949,23 @@
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="2:4">
-      <c r="B14" s="10" t="s">
+    <row r="14" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B14" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="11" t="s">
+      <c r="C14" s="4" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="15" spans="2:4">
-      <c r="B15" s="10" t="s">
+    <row r="15" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B15" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C15" s="11" t="s">
+      <c r="C15" s="4" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="16" spans="2:4" ht="75">
+    <row r="16" spans="2:4" ht="63.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B16" s="4" t="s">
         <v>25</v>
       </c>
@@ -828,185 +973,221 @@
         <v>26</v>
       </c>
     </row>
-    <row r="17" spans="2:3" ht="60">
+    <row r="17" spans="2:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="B17" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="C17" s="19" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="18" spans="2:3" ht="67.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B18" s="9" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="18" spans="2:3" ht="90">
-      <c r="B18" s="9" t="s">
+      <c r="C18" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="C18" s="4" t="s">
+    </row>
+    <row r="19" spans="2:3" ht="35.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B19" s="3" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="19" spans="2:3" ht="35.25" customHeight="1">
-      <c r="B19" s="3" t="s">
+      <c r="C19" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="C19" s="4" t="s">
+    </row>
+    <row r="20" spans="2:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="B20" s="17" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="20" spans="2:3" ht="30">
-      <c r="B20" s="3" t="s">
+      <c r="C20" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="C20" s="4" t="s">
+    </row>
+    <row r="21" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B21" s="17" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="21" spans="2:3" ht="30">
-      <c r="B21" s="3" t="s">
+      <c r="C21" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="C21" s="1" t="s">
+    </row>
+    <row r="22" spans="2:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="B22" s="3" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="22" spans="2:3" ht="33.75" customHeight="1">
-      <c r="B22" s="3" t="s">
+      <c r="C22" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C22" s="1" t="s">
+    </row>
+    <row r="23" spans="2:3" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B23" s="3" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="23" spans="2:3" ht="30">
-      <c r="B23" s="3" t="s">
+      <c r="C23" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C23" s="4" t="s">
+    </row>
+    <row r="24" spans="2:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="B24" s="3" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="24" spans="2:3" ht="45">
-      <c r="B24" s="3" t="s">
+      <c r="C24" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="C24" s="4" t="s">
+    </row>
+    <row r="25" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B25" s="3" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="25" spans="2:3" ht="45.75">
-      <c r="B25" s="3" t="s">
+      <c r="C25" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="C25" s="4" t="s">
+    </row>
+    <row r="26" spans="2:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="B26" s="3" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="26" spans="2:3">
-      <c r="B26" s="10" t="s">
+      <c r="C26" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="C26" s="12" t="s">
+    </row>
+    <row r="27" spans="2:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="B27" s="3" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="27" spans="2:3" ht="30">
-      <c r="B27" s="3" t="s">
+      <c r="C27" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="C27" s="4" t="s">
+    </row>
+    <row r="28" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B28" s="3" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="28" spans="2:3" ht="45">
-      <c r="B28" s="3" t="s">
+      <c r="C28" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="C28" s="4" t="s">
+    </row>
+    <row r="29" spans="2:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="B29" s="3" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="29" spans="2:3" ht="75">
-      <c r="B29" s="3" t="s">
+      <c r="C29" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="C29" s="4" t="s">
+    </row>
+    <row r="30" spans="2:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="B30" s="3" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="30" spans="2:3" ht="30">
-      <c r="B30" s="3" t="s">
+      <c r="C30" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="C30" s="4" t="s">
+    </row>
+    <row r="31" spans="2:3" ht="58" x14ac:dyDescent="0.35">
+      <c r="B31" s="3" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="31" spans="2:3" ht="30">
-      <c r="B31" s="3" t="s">
+      <c r="C31" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="C31" s="4" t="s">
+    </row>
+    <row r="32" spans="2:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="B32" s="3" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="32" spans="2:3" ht="45">
-      <c r="B32" s="4" t="s">
+      <c r="C32" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="C32" s="4" t="s">
+    </row>
+    <row r="33" spans="2:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="B33" s="3" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="33" spans="2:3" ht="75">
-      <c r="B33" s="3" t="s">
+      <c r="C33" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="C33" s="4" t="s">
+    </row>
+    <row r="34" spans="2:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="B34" s="4" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="34" spans="2:3" ht="60">
-      <c r="B34" s="4" t="s">
+      <c r="C34" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="C34" s="4" t="s">
+    </row>
+    <row r="35" spans="2:3" ht="58" x14ac:dyDescent="0.35">
+      <c r="B35" s="3" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="35" spans="2:3" ht="48" customHeight="1">
-      <c r="B35" s="3" t="s">
+      <c r="C35" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="C35" s="4" t="s">
+    </row>
+    <row r="36" spans="2:3" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="B36" s="4" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="36" spans="2:3" ht="30">
-      <c r="B36" s="3" t="s">
+      <c r="C36" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="C36" s="4" t="s">
+    </row>
+    <row r="37" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B37" s="3" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="37" spans="2:3" ht="63.75" customHeight="1">
-      <c r="B37" s="4" t="s">
+      <c r="C37" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="C37" s="4" t="s">
+    </row>
+    <row r="38" spans="2:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="B38" s="3" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="38" spans="2:3">
-      <c r="B38" s="3"/>
-      <c r="C38" s="3"/>
-    </row>
-    <row r="39" spans="2:3">
-      <c r="B39" s="3"/>
-      <c r="C39" s="3"/>
-    </row>
-    <row r="40" spans="2:3">
-      <c r="B40" s="3"/>
-      <c r="C40" s="3"/>
+      <c r="C38" s="4" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="39" spans="2:3" ht="63.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B39" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="40" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B40" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="C40" s="10" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="41" spans="2:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="B41" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="C41" s="11" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="42" spans="2:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="B42" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="C42" s="13" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="43" spans="2:3" ht="174" x14ac:dyDescent="0.35">
+      <c r="B43" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="C43" s="18" t="s">
+        <v>79</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1015,18 +1196,18 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1186,13 +1367,36 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{552932D6-818C-4E5F-A4DC-6AD4FB3E74DC}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CE224D68-DD8C-41E0-BC8F-161016676D5D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CE224D68-DD8C-41E0-BC8F-161016676D5D}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{552932D6-818C-4E5F-A4DC-6AD4FB3E74DC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{891F6E60-2DC7-4183-8443-781947774D29}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{891F6E60-2DC7-4183-8443-781947774D29}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="e01fda85-2bd3-4106-a425-b6fd761820cd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
update Excel KB, neues Wissen bzgl Sonderthemen-Störung Heizung/Strom
</commit_message>
<xml_diff>
--- a/Excels/Knowledge Base.xlsx
+++ b/Excels/Knowledge Base.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30613"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Zeyuan.Sun\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://itservicewn.sharepoint.com/sites/VODAFONEVIER/Freigegebene Dokumente/General/FAQ/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C97794A-0794-40C9-BE7B-FB1CC11B5996}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5430C901-FFE7-4B59-B31C-8A5A94D4034E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -124,6 +124,39 @@
   </si>
   <si>
     <t>Gasversorgung – Bioerdgas</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Anfragen zum Bezug von Bioerdgas/Biogas sowie zu einem benötigten Biogas-Nachweis müssen individuell durch den zuständigen Fachbereich geprüft werden. Dies betrifft beispielsweise die Frage, ob Bioerdgas über die Stadtwerke Waiblingen bezogen werden kann, wie ein Bezug möglich ist oder ob ein von einer Stadt bzw. Behörde geforderter Nachweis für Biogas ausgestellt werden kann. </t>
+    </r>
+    <r>
+      <rPr>
+        <strike/>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Schreiben Sie hierzu gerne eine E-Mail an vertrieb@stadtwerke-waiblingen.de oder bleiben sie in der Leitung, um mit einem Mitarbeiter verbunden zu werden.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (Kein Hinweis auf die E-Mailadresse geben).</t>
+    </r>
   </si>
   <si>
     <t>Lieferantenwechsel – Widerruf Fremdvertrag</t>
@@ -315,34 +348,19 @@
 Wenn Ihre Fernwärmeversorgung ausgefallen ist oder Sie eine andere Störung im Fernwärmenetz feststellen, melden Sie sich bitte unter 07151 131-501.
 Die Notfallnummern sind ausschließlich für Störungen im jeweiligen Versorgungsnetz vorgesehen.</t>
   </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Anfragen zum Bezug von Bioerdgas/Biogas sowie zu einem benötigten Biogas-Nachweis müssen individuell durch den zuständigen Fachbereich geprüft werden. Dies betrifft beispielsweise die Frage, ob Bioerdgas über die Stadtwerke Waiblingen bezogen werden kann, wie ein Bezug möglich ist oder ob ein von einer Stadt bzw. Behörde geforderter Nachweis für Biogas ausgestellt werden kann. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>(Kein Hinweis auf die E-Mailadresse geben).</t>
-    </r>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="11">
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -394,6 +412,14 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <strike/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -502,20 +528,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="2"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -528,16 +554,16 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -558,9 +584,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 – 2022-Design">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 – 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -598,7 +624,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 – 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -704,7 +730,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 – 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -846,7 +872,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -855,21 +881,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B2:D43"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="4.453125" customWidth="1"/>
-    <col min="2" max="2" width="43.26953125" customWidth="1"/>
-    <col min="3" max="3" width="170.1796875" customWidth="1"/>
+    <col min="1" max="1" width="4.42578125" customWidth="1"/>
+    <col min="2" max="2" width="43.28515625" customWidth="1"/>
+    <col min="3" max="3" width="170.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:4" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:4" ht="23.25" customHeight="1">
       <c r="B2" s="6" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="5"/>
       <c r="D2" s="7"/>
     </row>
-    <row r="4" spans="2:4" ht="26.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:4" ht="26.25" customHeight="1">
       <c r="B4" s="2" t="s">
         <v>1</v>
       </c>
@@ -877,7 +903,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="2:4" ht="29" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:4" ht="30">
       <c r="B5" s="3" t="s">
         <v>3</v>
       </c>
@@ -885,7 +911,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="2:4" ht="29" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:4" ht="30">
       <c r="B6" s="3" t="s">
         <v>5</v>
       </c>
@@ -893,7 +919,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="2:4" ht="29" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:4" ht="30">
       <c r="B7" s="3" t="s">
         <v>7</v>
       </c>
@@ -901,7 +927,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="2:4" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:4" ht="45">
       <c r="B8" s="3" t="s">
         <v>9</v>
       </c>
@@ -909,7 +935,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="2:4" ht="29" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:4" ht="30">
       <c r="B9" s="3" t="s">
         <v>11</v>
       </c>
@@ -917,7 +943,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:4">
       <c r="B10" s="3" t="s">
         <v>13</v>
       </c>
@@ -925,7 +951,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="11" spans="2:4" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:4" ht="45">
       <c r="B11" s="3" t="s">
         <v>15</v>
       </c>
@@ -933,7 +959,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="2:4" ht="29" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:4" ht="30">
       <c r="B12" s="3" t="s">
         <v>17</v>
       </c>
@@ -941,7 +967,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="13" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:4">
       <c r="B13" s="3" t="s">
         <v>19</v>
       </c>
@@ -949,7 +975,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:4">
       <c r="B14" s="3" t="s">
         <v>21</v>
       </c>
@@ -957,7 +983,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="15" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:4">
       <c r="B15" s="3" t="s">
         <v>23</v>
       </c>
@@ -965,7 +991,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="16" spans="2:4" ht="63.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:4" ht="63.75" customHeight="1">
       <c r="B16" s="4" t="s">
         <v>25</v>
       </c>
@@ -973,220 +999,220 @@
         <v>26</v>
       </c>
     </row>
-    <row r="17" spans="2:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:3" ht="60">
       <c r="B17" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="C17" s="19" t="s">
+      <c r="C17" s="17" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="18" spans="2:3" ht="67.5" customHeight="1">
+      <c r="B18" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="19" spans="2:3" ht="35.25" customHeight="1">
+      <c r="B19" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="20" spans="2:3" ht="45">
+      <c r="B20" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="C20" s="11" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="21" spans="2:3">
+      <c r="B21" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="C21" s="14" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="22" spans="2:3" ht="30">
+      <c r="B22" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="23" spans="2:3" ht="33.75" customHeight="1">
+      <c r="B23" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="24" spans="2:3" ht="30">
+      <c r="B24" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="25" spans="2:3">
+      <c r="B25" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C25" s="15" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="26" spans="2:3" ht="30">
+      <c r="B26" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="27" spans="2:3" ht="45">
+      <c r="B27" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="28" spans="2:3">
+      <c r="B28" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C28" s="16" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="29" spans="2:3" ht="30">
+      <c r="B29" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="30" spans="2:3" ht="30">
+      <c r="B30" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="31" spans="2:3" ht="60">
+      <c r="B31" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="32" spans="2:3" ht="30">
+      <c r="B32" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="33" spans="2:3" ht="30">
+      <c r="B33" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="34" spans="2:3" ht="30">
+      <c r="B34" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="35" spans="2:3" ht="60">
+      <c r="B35" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="36" spans="2:3" ht="45">
+      <c r="B36" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="37" spans="2:3" ht="48" customHeight="1">
+      <c r="B37" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="38" spans="2:3" ht="30">
+      <c r="B38" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="39" spans="2:3" ht="63.75" customHeight="1">
+      <c r="B39" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="40" spans="2:3">
+      <c r="B40" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="C40" s="10" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="41" spans="2:3" ht="30">
+      <c r="B41" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="C41" s="11" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="42" spans="2:3" ht="30">
+      <c r="B42" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="C42" s="13" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="43" spans="2:3" ht="180">
+      <c r="B43" s="19" t="s">
+        <v>79</v>
+      </c>
+      <c r="C43" s="19" t="s">
         <v>80</v>
-      </c>
-    </row>
-    <row r="18" spans="2:3" ht="67.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="19" spans="2:3" ht="35.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B19" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="20" spans="2:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="B20" s="17" t="s">
-        <v>32</v>
-      </c>
-      <c r="C20" s="11" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="21" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B21" s="17" t="s">
-        <v>34</v>
-      </c>
-      <c r="C21" s="14" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="22" spans="2:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="B22" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="23" spans="2:3" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B23" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="24" spans="2:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="B24" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="C24" s="4" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="25" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B25" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="C25" s="15" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="26" spans="2:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="B26" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="C26" s="4" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="27" spans="2:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="B27" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="C27" s="4" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="28" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B28" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="C28" s="16" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="29" spans="2:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="B29" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="C29" s="4" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="30" spans="2:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="B30" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="C30" s="4" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="31" spans="2:3" ht="58" x14ac:dyDescent="0.35">
-      <c r="B31" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="C31" s="4" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="32" spans="2:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="B32" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="C32" s="4" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="33" spans="2:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="B33" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="C33" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="34" spans="2:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="B34" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="C34" s="4" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="35" spans="2:3" ht="58" x14ac:dyDescent="0.35">
-      <c r="B35" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="C35" s="4" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="36" spans="2:3" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="B36" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="C36" s="4" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="37" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B37" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="C37" s="4" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="38" spans="2:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="B38" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="C38" s="4" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="39" spans="2:3" ht="63.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B39" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="C39" s="4" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="40" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B40" s="10" t="s">
-        <v>72</v>
-      </c>
-      <c r="C40" s="10" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="41" spans="2:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="B41" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="C41" s="11" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="42" spans="2:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="B42" s="12" t="s">
-        <v>76</v>
-      </c>
-      <c r="C42" s="13" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="43" spans="2:3" ht="174" x14ac:dyDescent="0.35">
-      <c r="B43" s="18" t="s">
-        <v>78</v>
-      </c>
-      <c r="C43" s="18" t="s">
-        <v>79</v>
       </c>
     </row>
   </sheetData>
@@ -1196,18 +1222,18 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1367,36 +1393,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CE224D68-DD8C-41E0-BC8F-161016676D5D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{552932D6-818C-4E5F-A4DC-6AD4FB3E74DC}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{552932D6-818C-4E5F-A4DC-6AD4FB3E74DC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CE224D68-DD8C-41E0-BC8F-161016676D5D}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{891F6E60-2DC7-4183-8443-781947774D29}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="e01fda85-2bd3-4106-a425-b6fd761820cd"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{891F6E60-2DC7-4183-8443-781947774D29}"/>
 </file>
</xml_diff>